<commit_message>
almost finish the readme
</commit_message>
<xml_diff>
--- a/exe2/output_features/Unified_Top_Features.xlsx
+++ b/exe2/output_features/Unified_Top_Features.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elino\Desktop\לימודים\שנה ד\סמסטר א\איחזור מידע\ex\ir\exe2\output_features\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978B5725-5ED7-4036-A04C-17ACD4D6650D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{134139FB-8BD1-4FF5-AC70-F399DCB7D94B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Class_0_Features" sheetId="1" r:id="rId1"/>
@@ -353,12 +353,108 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB7FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -388,12 +484,60 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -402,6 +546,12 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFB7FF"/>
+      <color rgb="FFFF66FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -740,19 +890,19 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2">
         <v>5.885919460251281</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="2">
         <v>8.6398386844989579E-3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="2">
@@ -766,19 +916,19 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>5.7542568173102646</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D3" s="2">
         <v>8.6329546873103458E-3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="8" t="s">
         <v>28</v>
       </c>
       <c r="F3" s="2">
@@ -792,7 +942,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="2">
@@ -804,7 +954,7 @@
       <c r="D4" s="2">
         <v>8.5512001101180415E-3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F4" s="2">
@@ -824,7 +974,7 @@
       <c r="B5" s="2">
         <v>5.5537676302921124</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="2">
@@ -934,7 +1084,7 @@
       <c r="D9" s="2">
         <v>7.3697717789353214E-3</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="F9" s="2">
@@ -1084,7 +1234,7 @@
       <c r="B15" s="2">
         <v>5.2619450961110044</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="2">
@@ -1142,7 +1292,7 @@
       <c r="D17" s="2">
         <v>6.6421170424737176E-3</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="10" t="s">
         <v>41</v>
       </c>
       <c r="F17" s="2">
@@ -1162,7 +1312,7 @@
       <c r="B18" s="2">
         <v>5.2303038939434181</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="10" t="s">
         <v>41</v>
       </c>
       <c r="D18" s="2">
@@ -1194,7 +1344,7 @@
       <c r="D19" s="2">
         <v>6.5886471512937271E-3</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="7" t="s">
         <v>54</v>
       </c>
       <c r="F19" s="2">
@@ -1214,7 +1364,7 @@
       <c r="B20" s="2">
         <v>5.2153105459766991</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="9" t="s">
         <v>43</v>
       </c>
       <c r="D20" s="2">
@@ -1246,13 +1396,13 @@
       <c r="D21" s="2">
         <v>6.5053188861994536E-3</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="9" t="s">
         <v>43</v>
       </c>
       <c r="F21" s="2">
         <v>1.712699899055832E-2</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="7" t="s">
         <v>54</v>
       </c>
       <c r="H21" s="2">
@@ -1315,7 +1465,7 @@
       <c r="B2" s="2">
         <v>6.7081395104597696</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="7" t="s">
         <v>74</v>
       </c>
       <c r="D2" s="2">
@@ -1327,7 +1477,7 @@
       <c r="F2" s="2">
         <v>0.13399544720151349</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="12" t="s">
         <v>56</v>
       </c>
       <c r="H2" s="2">
@@ -1335,7 +1485,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="5" t="s">
         <v>63</v>
       </c>
       <c r="B3" s="2">
@@ -1353,7 +1503,7 @@
       <c r="F3" s="2">
         <v>0.1128480740311532</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="14" t="s">
         <v>57</v>
       </c>
       <c r="H3" s="2">
@@ -1361,19 +1511,19 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="7" t="s">
         <v>74</v>
       </c>
       <c r="B4" s="2">
         <v>6.6849731084261954</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="18" t="s">
         <v>67</v>
       </c>
       <c r="D4" s="2">
         <v>4.0838513248579997E-2</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="7" t="s">
         <v>74</v>
       </c>
       <c r="F4" s="2">
@@ -1387,13 +1537,13 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="17" t="s">
         <v>75</v>
       </c>
       <c r="B5" s="2">
         <v>6.6803912450810889</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="17" t="s">
         <v>75</v>
       </c>
       <c r="D5" s="2">
@@ -1405,7 +1555,7 @@
       <c r="F5" s="2">
         <v>0.1102758688646634</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="10" t="s">
         <v>59</v>
       </c>
       <c r="H5" s="2">
@@ -1413,25 +1563,25 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="18" t="s">
         <v>67</v>
       </c>
       <c r="B6" s="2">
         <v>6.6803073997788482</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>61</v>
       </c>
       <c r="D6" s="2">
         <v>4.0321708782592253E-2</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="17" t="s">
         <v>75</v>
       </c>
       <c r="F6" s="2">
         <v>0.108799907044846</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="11" t="s">
         <v>60</v>
       </c>
       <c r="H6" s="2">
@@ -1445,7 +1595,7 @@
       <c r="B7" s="2">
         <v>6.6767904181217226</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="12" t="s">
         <v>56</v>
       </c>
       <c r="D7" s="2">
@@ -1457,7 +1607,7 @@
       <c r="F7" s="2">
         <v>0.10879969576539029</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="4" t="s">
         <v>61</v>
       </c>
       <c r="H7" s="2">
@@ -1465,19 +1615,19 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="11" t="s">
         <v>60</v>
       </c>
       <c r="B8" s="2">
         <v>6.641124804383244</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="11" t="s">
         <v>60</v>
       </c>
       <c r="D8" s="2">
         <v>3.8173467190997762E-2</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="11" t="s">
         <v>60</v>
       </c>
       <c r="F8" s="2">
@@ -1491,25 +1641,25 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="9" t="s">
         <v>71</v>
       </c>
       <c r="B9" s="2">
         <v>6.6295584920296902</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="13" t="s">
         <v>77</v>
       </c>
       <c r="D9" s="2">
         <v>3.6868570981199777E-2</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="13" t="s">
         <v>77</v>
       </c>
       <c r="F9" s="2">
         <v>9.7004267171879682E-2</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="5" t="s">
         <v>63</v>
       </c>
       <c r="H9" s="2">
@@ -1517,19 +1667,19 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="13" t="s">
         <v>77</v>
       </c>
       <c r="B10" s="2">
         <v>6.6295440805321491</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="9" t="s">
         <v>71</v>
       </c>
       <c r="D10" s="2">
         <v>3.6733548009058627E-2</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="9" t="s">
         <v>71</v>
       </c>
       <c r="F10" s="2">
@@ -1575,7 +1725,7 @@
       <c r="B12" s="2">
         <v>6.4363004972538391</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="10" t="s">
         <v>59</v>
       </c>
       <c r="D12" s="2">
@@ -1607,7 +1757,7 @@
       <c r="D13" s="2">
         <v>3.6220535370372557E-2</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="4" t="s">
         <v>61</v>
       </c>
       <c r="F13" s="2">
@@ -1621,19 +1771,19 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="16" t="s">
         <v>81</v>
       </c>
       <c r="B14" s="2">
         <v>6.3786149034950839</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="15" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="2">
         <v>3.6045844625495538E-2</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F14" s="2">
@@ -1659,13 +1809,13 @@
       <c r="D15" s="2">
         <v>3.5897732989010833E-2</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="15" t="s">
         <v>62</v>
       </c>
       <c r="F15" s="2">
         <v>8.1962186455116506E-2</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="18" t="s">
         <v>67</v>
       </c>
       <c r="H15" s="2">
@@ -1679,7 +1829,7 @@
       <c r="B16" s="2">
         <v>6.3186680919090588</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="14" t="s">
         <v>57</v>
       </c>
       <c r="D16" s="2">
@@ -1763,13 +1913,13 @@
       <c r="D19" s="2">
         <v>3.2727071208447388E-2</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="16" t="s">
         <v>81</v>
       </c>
       <c r="F19" s="2">
         <v>6.8574755047217981E-2</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="9" t="s">
         <v>71</v>
       </c>
       <c r="H19" s="2">

</xml_diff>